<commit_message>
feat: atualizar vendas recuperadas do pwr e adicionar auto-push no robo de varredura
</commit_message>
<xml_diff>
--- a/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-09-13).xlsx
+++ b/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-09-13).xlsx
@@ -935,13 +935,13 @@
     <t>214</t>
   </si>
   <si>
-    <t>29</t>
-  </si>
-  <si>
-    <t>R$ 9.033,52</t>
-  </si>
-  <si>
-    <t>99.0</t>
+    <t>28</t>
+  </si>
+  <si>
+    <t>R$ 9.012,32</t>
+  </si>
+  <si>
+    <t>98.8</t>
   </si>
   <si>
     <t>65.6</t>
@@ -953,13 +953,13 @@
     <t>21.9</t>
   </si>
   <si>
-    <t>8.6</t>
+    <t>8.7</t>
   </si>
   <si>
     <t>6.1</t>
   </si>
   <si>
-    <t>32.0%</t>
+    <t>32.1%</t>
   </si>
   <si>
     <t>17.5%</t>
@@ -7613,7 +7613,7 @@
         <v>19579</v>
       </c>
       <c r="B42" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C42" s="4">
         <v>51</v>
@@ -7643,14 +7643,26 @@
         <v>58</v>
       </c>
       <c r="L42" s="4"/>
-      <c r="M42" s="5"/>
-      <c r="N42" s="6"/>
+      <c r="M42" s="5">
+        <v>5111.9300000000003</v>
+      </c>
+      <c r="N42" s="6">
+        <v>63</v>
+      </c>
       <c r="O42" s="6"/>
-      <c r="P42" s="7"/>
-      <c r="Q42" s="8"/>
-      <c r="R42" s="8"/>
+      <c r="P42" s="7">
+        <v>6.7954306451612911</v>
+      </c>
+      <c r="Q42" s="8">
+        <v>23.158805660377357</v>
+      </c>
+      <c r="R42" s="8">
+        <v>10.489795918367347</v>
+      </c>
       <c r="S42" s="8"/>
-      <c r="T42" s="9"/>
+      <c r="T42" s="9">
+        <v>0.18867924528301888</v>
+      </c>
       <c r="U42" s="9"/>
       <c r="V42" s="9"/>
       <c r="W42" s="9"/>

</xml_diff>